<commit_message>
Revise EXW pricing with Almaty local market anchors
Add Almaty retail neon price benchmarks (KZT) and lower the recommended
project EXW from USD 7.20 to USD 6.20/m so the partner retains landed
margin against local mid-tier shelf prices.

Co-authored-by: OSEEEEEEEE <OSEEEEEEEE@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/MIHORAY_EXW定价建议_RFQ20260916核查.xlsx
+++ b/MIHORAY_EXW定价建议_RFQ20260916核查.xlsx
@@ -7,9 +7,11 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="报价合理性核查" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="EXW建议报价_MIHORAY" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="原报价vs建议对照" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="阿拉木图市场对照" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="修订EXW_含本地市场" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="报价合理性核查" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="EXW建议报价_MIHORAY" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="原报价vs建议对照" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -19,7 +21,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="17">
+  <fonts count="18">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -109,6 +111,12 @@
       <color rgb="00888888"/>
       <sz val="8"/>
     </font>
+    <font>
+      <name val="微软雅黑"/>
+      <b val="1"/>
+      <color rgb="001F3A5F"/>
+      <sz val="14"/>
+    </font>
   </fonts>
   <fills count="10">
     <fill>
@@ -158,7 +166,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="6">
     <border>
       <left/>
       <right/>
@@ -180,11 +188,55 @@
         <color rgb="00B0B0B0"/>
       </bottom>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="00B0B0B0"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00B0B0B0"/>
+      </right>
+      <top style="thin">
+        <color rgb="00B0B0B0"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="00B0B0B0"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00B0B0B0"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00B0B0B0"/>
+      </right>
+      <top style="thin">
+        <color rgb="00B0B0B0"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00B0B0B0"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="36">
+  <cellXfs count="48">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -249,6 +301,28 @@
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="6" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="8" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -614,6 +688,956 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:F41"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="34" customWidth="1" min="1" max="1"/>
+    <col width="18" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="14" customWidth="1" min="5" max="5"/>
+    <col width="42" customWidth="1" min="6" max="6"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="36" t="inlineStr">
+        <is>
+          <t>阿拉木图本地市场价核对 · 对 EXW 建议的修正</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="36" customHeight="1">
+      <c r="A2" s="8" t="inlineStr">
+        <is>
+          <t>核查日期：2026-09-18｜汇率参考：1 USD ≈ 445 KZT（哈萨克斯坦国家银行 2026-09-17 约 444.88）｜说明：此前建议偏重成本/品牌，本地零售锚点不足，本表补齐</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="3" t="inlineStr">
+        <is>
+          <t>一、直接回答</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="56" customHeight="1">
+      <c r="A5" s="13" t="inlineStr">
+        <is>
+          <t>之前那版 EXW USD 7.20/m 没有充分按阿拉木图零售行情校准。对照本地中档硅胶/建筑级霓虹零售约 2,500–3,500₸/m（≈USD 5.6–7.9，已含进口与本地加价），对本地合作伙伴来说 7.20 EXW 略偏高、可谈空间偏紧；但原报价 ¥17（≈USD 2.36）仍然过低。修正后推荐项目 EXW：USD 6.20/m。</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="3" t="inlineStr">
+        <is>
+          <t>二、阿拉木图公开零售价（2026-09 检索）</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="5" t="inlineStr">
+        <is>
+          <t>本地产品（公开价）</t>
+        </is>
+      </c>
+      <c r="B8" s="5" t="inlineStr">
+        <is>
+          <t>规格层级</t>
+        </is>
+      </c>
+      <c r="C8" s="5" t="inlineStr">
+        <is>
+          <t>₸/m</t>
+        </is>
+      </c>
+      <c r="D8" s="5" t="inlineStr">
+        <is>
+          <t>≈USD/m</t>
+        </is>
+      </c>
+      <c r="E8" s="5" t="inlineStr">
+        <is>
+          <t>来源类型</t>
+        </is>
+      </c>
+      <c r="F8" s="5" t="inlineStr">
+        <is>
+          <t>与本项目相关性</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="28" customHeight="1">
+      <c r="A9" s="7" t="inlineStr">
+        <is>
+          <t>柔性霓虹/冷氖 8×16 220V</t>
+        </is>
+      </c>
+      <c r="B9" s="7" t="inlineStr">
+        <is>
+          <t>低端广告字/现货</t>
+        </is>
+      </c>
+      <c r="C9" s="7" t="n">
+        <v>980</v>
+      </c>
+      <c r="D9" s="7" t="n">
+        <v>2.2</v>
+      </c>
+      <c r="E9" s="7" t="inlineStr">
+        <is>
+          <t>Flagma.kz 阿拉木图</t>
+        </is>
+      </c>
+      <c r="F9" s="7" t="inlineStr">
+        <is>
+          <t>低：PVC高压，非48V项目级</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="28" customHeight="1">
+      <c r="A10" s="7" t="inlineStr">
+        <is>
+          <t>Flex Neon 10×5 12V</t>
+        </is>
+      </c>
+      <c r="B10" s="7" t="inlineStr">
+        <is>
+          <t>低端装饰现货</t>
+        </is>
+      </c>
+      <c r="C10" s="7" t="n">
+        <v>1147</v>
+      </c>
+      <c r="D10" s="7" t="n">
+        <v>2.58</v>
+      </c>
+      <c r="E10" s="7" t="inlineStr">
+        <is>
+          <t>Satu.kz / 本地商户</t>
+        </is>
+      </c>
+      <c r="F10" s="7" t="inlineStr">
+        <is>
+          <t>低</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="28" customHeight="1">
+      <c r="A11" s="7" t="inlineStr">
+        <is>
+          <t>硅胶霓虹 8×16 12V</t>
+        </is>
+      </c>
+      <c r="B11" s="7" t="inlineStr">
+        <is>
+          <t>中低端硅胶现货</t>
+        </is>
+      </c>
+      <c r="C11" s="7" t="n">
+        <v>1800</v>
+      </c>
+      <c r="D11" s="7" t="n">
+        <v>4.04</v>
+      </c>
+      <c r="E11" s="7" t="inlineStr">
+        <is>
+          <t>LedProStore 阿拉木图</t>
+        </is>
+      </c>
+      <c r="F11" s="7" t="inlineStr">
+        <is>
+          <t>中低：同截面但12V短回路</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="28" customHeight="1">
+      <c r="A12" s="12" t="inlineStr">
+        <is>
+          <t>建筑级 Flex 10W IP67 220V</t>
+        </is>
+      </c>
+      <c r="B12" s="12" t="inlineStr">
+        <is>
+          <t>中档立面现货</t>
+        </is>
+      </c>
+      <c r="C12" s="12" t="n">
+        <v>2500</v>
+      </c>
+      <c r="D12" s="12" t="n">
+        <v>5.62</v>
+      </c>
+      <c r="E12" s="12" t="inlineStr">
+        <is>
+          <t>INTERMIR 阿拉木图</t>
+        </is>
+      </c>
+      <c r="F12" s="12" t="inlineStr">
+        <is>
+          <t>中：立面用途，非48V定制</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="28" customHeight="1">
+      <c r="A13" s="12" t="inlineStr">
+        <is>
+          <t>硅胶方型 20×20 24V IP67</t>
+        </is>
+      </c>
+      <c r="B13" s="12" t="inlineStr">
+        <is>
+          <t>中高档硅胶现货</t>
+        </is>
+      </c>
+      <c r="C13" s="12" t="n">
+        <v>3500</v>
+      </c>
+      <c r="D13" s="12" t="n">
+        <v>7.87</v>
+      </c>
+      <c r="E13" s="12" t="inlineStr">
+        <is>
+          <t>LedProStore 阿拉木图</t>
+        </is>
+      </c>
+      <c r="F13" s="12" t="inlineStr">
+        <is>
+          <t>高：最接近的本地硅胶锚点</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="40" customHeight="1">
+      <c r="A15" s="8" t="inlineStr">
+        <is>
+          <t>本地公开价带结论：低端现货 ≈ USD 2.2–4.0/m；中档立面/硅胶零售 ≈ USD 5.6–7.9/m（到货+本地毛利后的卖价，不是中国EXW）。未检索到同规格「48V / 30m单回路 / CRI90 项目定制」的公开标价——该类多为工程询价。</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="3" t="inlineStr">
+        <is>
+          <t>三、价格锚点对比（8×16 主推）</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="11" t="inlineStr">
+        <is>
+          <t>锚点</t>
+        </is>
+      </c>
+      <c r="B18" s="11" t="inlineStr">
+        <is>
+          <t>USD/m</t>
+        </is>
+      </c>
+      <c r="C18" s="11" t="inlineStr">
+        <is>
+          <t>约合₸/m</t>
+        </is>
+      </c>
+      <c r="D18" s="11" t="inlineStr">
+        <is>
+          <t>角色</t>
+        </is>
+      </c>
+      <c r="E18" s="11" t="inlineStr">
+        <is>
+          <t>评价</t>
+        </is>
+      </c>
+      <c r="F18" s="11" t="inlineStr"/>
+    </row>
+    <row r="19" ht="26" customHeight="1">
+      <c r="A19" s="37" t="inlineStr">
+        <is>
+          <t>原内部报价 ¥17</t>
+        </is>
+      </c>
+      <c r="B19" s="37" t="n">
+        <v>2.36</v>
+      </c>
+      <c r="C19" s="37" t="n">
+        <v>1051</v>
+      </c>
+      <c r="D19" s="37" t="inlineStr">
+        <is>
+          <t>中国成本导向</t>
+        </is>
+      </c>
+      <c r="E19" s="37" t="inlineStr">
+        <is>
+          <t>过低，低于本地低端零售逻辑混乱</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="26" customHeight="1">
+      <c r="A20" s="38" t="inlineStr">
+        <is>
+          <t>阿拉木图中档零售</t>
+        </is>
+      </c>
+      <c r="B20" s="38" t="n">
+        <v>5.6</v>
+      </c>
+      <c r="C20" s="38" t="n">
+        <v>2500</v>
+      </c>
+      <c r="D20" s="38" t="inlineStr">
+        <is>
+          <t>本地现货卖价</t>
+        </is>
+      </c>
+      <c r="E20" s="38" t="inlineStr">
+        <is>
+          <t>含进口与本地加价的货架价</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="26" customHeight="1">
+      <c r="A21" s="38" t="inlineStr">
+        <is>
+          <t>阿拉木图硅胶中高档零售</t>
+        </is>
+      </c>
+      <c r="B21" s="38" t="n">
+        <v>7.9</v>
+      </c>
+      <c r="C21" s="38" t="n">
+        <v>3500</v>
+      </c>
+      <c r="D21" s="38" t="inlineStr">
+        <is>
+          <t>本地硅胶卖价</t>
+        </is>
+      </c>
+      <c r="E21" s="38" t="inlineStr">
+        <is>
+          <t>最接近的货架上限锚点</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="26" customHeight="1">
+      <c r="A22" s="39" t="inlineStr">
+        <is>
+          <t>前版建议 EXW 7.20</t>
+        </is>
+      </c>
+      <c r="B22" s="39" t="n">
+        <v>7.2</v>
+      </c>
+      <c r="C22" s="39" t="n">
+        <v>3204</v>
+      </c>
+      <c r="D22" s="39" t="inlineStr">
+        <is>
+          <t>中国出厂给伙伴</t>
+        </is>
+      </c>
+      <c r="E22" s="39" t="inlineStr">
+        <is>
+          <t>接近甚至高于本地中高档零售，伙伴加价空间紧</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="26" customHeight="1">
+      <c r="A23" s="40" t="inlineStr">
+        <is>
+          <t>修正建议 EXW 6.20</t>
+        </is>
+      </c>
+      <c r="B23" s="40" t="n">
+        <v>6.2</v>
+      </c>
+      <c r="C23" s="40" t="n">
+        <v>2759</v>
+      </c>
+      <c r="D23" s="40" t="inlineStr">
+        <is>
+          <t>推荐项目出厂价</t>
+        </is>
+      </c>
+      <c r="E23" s="40" t="inlineStr">
+        <is>
+          <t>给伙伴留出落地+毛利空间，仍高于白牌</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="26" customHeight="1">
+      <c r="A24" s="38" t="inlineStr">
+        <is>
+          <t>伙伴落地后预估卖给项目</t>
+        </is>
+      </c>
+      <c r="B24" s="38" t="n">
+        <v>10.5</v>
+      </c>
+      <c r="C24" s="38" t="n">
+        <v>4672</v>
+      </c>
+      <c r="D24" s="38" t="inlineStr">
+        <is>
+          <t>工程销售价</t>
+        </is>
+      </c>
+      <c r="E24" s="38" t="inlineStr">
+        <is>
+          <t>高于本地现货，但对标Philips方案仍有优势</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="3" t="inlineStr">
+        <is>
+          <t>四、伙伴侧落地成本粗算（阿拉木图，示意）</t>
+        </is>
+      </c>
+    </row>
+    <row r="27" ht="56" customHeight="1">
+      <c r="A27" s="41" t="inlineStr">
+        <is>
+          <t>EXW 6.20 + 运杂约 0.80–1.20 + 清关/VAT等约 1.00–1.40 ≈ 落地 USD 8.0–8.8/m（约 3,560–3,920₸）。伙伴再加 25–35% 工程毛利 → 报给商业中心约 USD 10–12/m（约 4,450–5,340₸）。相对本地 2,500–3,500₸ 现货贵一截，但可用「48V长回路、室内电源、DALI、CRI90、2年项目质保、替代Philips 24V立面方案」解释溢价。</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="10" t="inlineStr">
+        <is>
+          <t>五、修正后的 EXW 建议（含本地市场）</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="11" t="inlineStr">
+        <is>
+          <t>档位</t>
+        </is>
+      </c>
+      <c r="B30" s="11" t="inlineStr">
+        <is>
+          <t>8×16 EXW</t>
+        </is>
+      </c>
+      <c r="C30" s="11" t="inlineStr">
+        <is>
+          <t>约合₸ EXW</t>
+        </is>
+      </c>
+      <c r="D30" s="11" t="inlineStr">
+        <is>
+          <t>何时用</t>
+        </is>
+      </c>
+      <c r="E30" s="11" t="inlineStr">
+        <is>
+          <t>相对本地市场</t>
+        </is>
+      </c>
+      <c r="F30" s="11" t="inlineStr"/>
+    </row>
+    <row r="31">
+      <c r="A31" s="14" t="inlineStr">
+        <is>
+          <t>清单价 List</t>
+        </is>
+      </c>
+      <c r="B31" s="14" t="inlineStr">
+        <is>
+          <t>USD 7.20</t>
+        </is>
+      </c>
+      <c r="C31" s="14" t="inlineStr">
+        <is>
+          <t>3204₸</t>
+        </is>
+      </c>
+      <c r="D31" s="14" t="inlineStr">
+        <is>
+          <t>无本地竞争压力/强调品牌时</t>
+        </is>
+      </c>
+      <c r="E31" s="14" t="inlineStr">
+        <is>
+          <t>偏高，需强依赖Philips对比话术</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="42" t="inlineStr">
+        <is>
+          <t>项目价 Project（推荐）</t>
+        </is>
+      </c>
+      <c r="B32" s="42" t="inlineStr">
+        <is>
+          <t>USD 6.20</t>
+        </is>
+      </c>
+      <c r="C32" s="42" t="inlineStr">
+        <is>
+          <t>2759₸</t>
+        </is>
+      </c>
+      <c r="D32" s="42" t="inlineStr">
+        <is>
+          <t>阿拉木图本项目正式报价</t>
+        </is>
+      </c>
+      <c r="E32" s="42" t="inlineStr">
+        <is>
+          <t>平衡品牌、售后与伙伴加价空间</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="14" t="inlineStr">
+        <is>
+          <t>战略价 Partner</t>
+        </is>
+      </c>
+      <c r="B33" s="14" t="inlineStr">
+        <is>
+          <t>USD 5.60</t>
+        </is>
+      </c>
+      <c r="C33" s="14" t="inlineStr">
+        <is>
+          <t>2492₸</t>
+        </is>
+      </c>
+      <c r="D33" s="14" t="inlineStr">
+        <is>
+          <t>量大或长期代理</t>
+        </is>
+      </c>
+      <c r="E33" s="14" t="inlineStr">
+        <is>
+          <t>接近本地中档零售对应的出厂下限</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="43" t="inlineStr">
+        <is>
+          <t>底线 Floor</t>
+        </is>
+      </c>
+      <c r="B34" s="43" t="inlineStr">
+        <is>
+          <t>USD 5.20</t>
+        </is>
+      </c>
+      <c r="C34" s="43" t="inlineStr">
+        <is>
+          <t>2314₸</t>
+        </is>
+      </c>
+      <c r="D34" s="43" t="inlineStr">
+        <is>
+          <t>仅大单且压缩服务范围</t>
+        </is>
+      </c>
+      <c r="E34" s="43" t="inlineStr">
+        <is>
+          <t>再低进入白牌肉搏，不建议</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="44" t="inlineStr">
+        <is>
+          <t>10×20 同步修正：项目价 USD 8.00/m（前版 9.20 对本地偏高）；战略价 7.20；清单价 8.80。</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="3" t="inlineStr">
+        <is>
+          <t>六、与 Philips 原设计的关系（本地决策逻辑）</t>
+        </is>
+      </c>
+    </row>
+    <row r="39" ht="56" customHeight="1">
+      <c r="A39" s="41" t="inlineStr">
+        <is>
+          <t>客户原方案是 Philips 24V 立面系统；哈萨克斯坦有 Signify/Philips 工程渠道，但公开零售几乎看不到同级单价（工程报价制）。商业中心比的是「整包可靠性/维保/电源位置」，不是 Satu 上的 1,800₸ 霓虹。因此：不要按低端现货去打价格战；也不宜 EXW 报到接近本地中高档零售（7.2），以免伙伴无利可图。6.20 是把本地货架价、品牌调性、售后准备金和伙伴加价一起折中后的数。</t>
+        </is>
+      </c>
+    </row>
+    <row r="41" ht="36" customHeight="1">
+      <c r="A41" s="8" t="inlineStr">
+        <is>
+          <t>来源摘录：INTERMIR 2,500₸/m；LedProStore 8×16 12V 1,800₸/m、20×20 24V 3,500₸/m；Flagma 约 980₸/m；汇率 NBK 2026-09-17。本地价会变动，签约前建议伙伴再扫一眼货架竞品。</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="14">
+    <mergeCell ref="A38:F38"/>
+    <mergeCell ref="A2:F2"/>
+    <mergeCell ref="A41:F41"/>
+    <mergeCell ref="A36:F36"/>
+    <mergeCell ref="A1:F1"/>
+    <mergeCell ref="A5:F5"/>
+    <mergeCell ref="A29:F29"/>
+    <mergeCell ref="A27:F27"/>
+    <mergeCell ref="A17:F17"/>
+    <mergeCell ref="A4:F4"/>
+    <mergeCell ref="A26:F26"/>
+    <mergeCell ref="A39:F39"/>
+    <mergeCell ref="A15:F15"/>
+    <mergeCell ref="A7:F7"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:G15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="6" customWidth="1" min="1" max="1"/>
+    <col width="50" customWidth="1" min="2" max="2"/>
+    <col width="10" customWidth="1" min="3" max="3"/>
+    <col width="8" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="12" customWidth="1" min="6" max="6"/>
+    <col width="14" customWidth="1" min="7" max="7"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="17" t="inlineStr">
+        <is>
+          <t>MIHORAY EXW Quotation — REVISED with Almaty market check</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="19" t="inlineStr">
+        <is>
+          <t>Quote No.: MIH-ALM-20260918-03 | Date: 2026-09-18 | EXW Jiangmen | Valid 15 days | Replaces prior USD7.20 recommendation for this market</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="45" t="inlineStr">
+        <is>
+          <t>Item</t>
+        </is>
+      </c>
+      <c r="B4" s="45" t="inlineStr">
+        <is>
+          <t>Product Description</t>
+        </is>
+      </c>
+      <c r="C4" s="45" t="inlineStr">
+        <is>
+          <t>Qty</t>
+        </is>
+      </c>
+      <c r="D4" s="45" t="inlineStr">
+        <is>
+          <t>Unit</t>
+        </is>
+      </c>
+      <c r="E4" s="45" t="inlineStr">
+        <is>
+          <t>Unit Price($)</t>
+        </is>
+      </c>
+      <c r="F4" s="45" t="inlineStr">
+        <is>
+          <t>Amount($)</t>
+        </is>
+      </c>
+      <c r="G4" s="45" t="inlineStr">
+        <is>
+          <t>Lead time</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="58" customHeight="1">
+      <c r="A5" s="22" t="n">
+        <v>1</v>
+      </c>
+      <c r="B5" s="23" t="inlineStr">
+        <is>
+          <t>MIHORAY Architectural Silicone Neon 8×16mm | DC48V | 10W/m | 3000K | CRI≥90 | IP65/67
+Up to 30m/circuit | 10m modules | Project QA + 2yr warranty reserve
+Almaty-market revised project EXW (was 7.20 draft)</t>
+        </is>
+      </c>
+      <c r="C5" s="22" t="n">
+        <v>30</v>
+      </c>
+      <c r="D5" s="22" t="inlineStr">
+        <is>
+          <t>m</t>
+        </is>
+      </c>
+      <c r="E5" s="22" t="n">
+        <v>6.2</v>
+      </c>
+      <c r="F5" s="22" t="n">
+        <v>186</v>
+      </c>
+      <c r="G5" s="22" t="inlineStr">
+        <is>
+          <t>15-25 WDs</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="28" customHeight="1">
+      <c r="A6" s="24" t="n">
+        <v>2</v>
+      </c>
+      <c r="B6" s="25" t="inlineStr">
+        <is>
+          <t>Option: 10×20mm same electrical family (thicker facade line)</t>
+        </is>
+      </c>
+      <c r="C6" s="24" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="D6" s="24" t="inlineStr">
+        <is>
+          <t>m</t>
+        </is>
+      </c>
+      <c r="E6" s="24" t="n">
+        <v>8</v>
+      </c>
+      <c r="F6" s="24" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G6" s="24" t="inlineStr">
+        <is>
+          <t>15-25 WDs</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="28" customHeight="1">
+      <c r="A7" s="24" t="n">
+        <v>3</v>
+      </c>
+      <c r="B7" s="25" t="inlineStr">
+        <is>
+          <t>Seamless mid-joint kit for 10m modules</t>
+        </is>
+      </c>
+      <c r="C7" s="24" t="n">
+        <v>2</v>
+      </c>
+      <c r="D7" s="24" t="inlineStr">
+        <is>
+          <t>set</t>
+        </is>
+      </c>
+      <c r="E7" s="24" t="n">
+        <v>1.6</v>
+      </c>
+      <c r="F7" s="24" t="n">
+        <v>3.2</v>
+      </c>
+      <c r="G7" s="24" t="inlineStr">
+        <is>
+          <t>with neon</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="28" customHeight="1">
+      <c r="A8" s="24" t="n">
+        <v>4</v>
+      </c>
+      <c r="B8" s="25" t="inlineStr">
+        <is>
+          <t>Front cable entry kit 30cm</t>
+        </is>
+      </c>
+      <c r="C8" s="24" t="n">
+        <v>1</v>
+      </c>
+      <c r="D8" s="24" t="inlineStr">
+        <is>
+          <t>set</t>
+        </is>
+      </c>
+      <c r="E8" s="24" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="F8" s="24" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="G8" s="24" t="inlineStr">
+        <is>
+          <t>with neon</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="28" customHeight="1">
+      <c r="A9" s="24" t="n">
+        <v>5</v>
+      </c>
+      <c r="B9" s="25" t="inlineStr">
+        <is>
+          <t>End cap potted</t>
+        </is>
+      </c>
+      <c r="C9" s="24" t="n">
+        <v>1</v>
+      </c>
+      <c r="D9" s="24" t="inlineStr">
+        <is>
+          <t>pc</t>
+        </is>
+      </c>
+      <c r="E9" s="24" t="n">
+        <v>0.16</v>
+      </c>
+      <c r="F9" s="24" t="n">
+        <v>0.16</v>
+      </c>
+      <c r="G9" s="24" t="inlineStr">
+        <is>
+          <t>with neon</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="28" customHeight="1">
+      <c r="A10" s="24" t="n">
+        <v>6</v>
+      </c>
+      <c r="B10" s="25" t="inlineStr">
+        <is>
+          <t>Aluminum profile 8×16 /m</t>
+        </is>
+      </c>
+      <c r="C10" s="24" t="n">
+        <v>30</v>
+      </c>
+      <c r="D10" s="24" t="inlineStr">
+        <is>
+          <t>m</t>
+        </is>
+      </c>
+      <c r="E10" s="24" t="n">
+        <v>0.95</v>
+      </c>
+      <c r="F10" s="24" t="n">
+        <v>28.5</v>
+      </c>
+      <c r="G10" s="24" t="inlineStr">
+        <is>
+          <t>with neon</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="28" customHeight="1">
+      <c r="A11" s="24" t="n">
+        <v>7</v>
+      </c>
+      <c r="B11" s="25" t="inlineStr">
+        <is>
+          <t>Fixing clip</t>
+        </is>
+      </c>
+      <c r="C11" s="24" t="n">
+        <v>120</v>
+      </c>
+      <c r="D11" s="24" t="inlineStr">
+        <is>
+          <t>pc</t>
+        </is>
+      </c>
+      <c r="E11" s="24" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="F11" s="24" t="n">
+        <v>12</v>
+      </c>
+      <c r="G11" s="24" t="inlineStr">
+        <is>
+          <t>with neon</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="28" customHeight="1">
+      <c r="A12" s="24" t="n">
+        <v>8</v>
+      </c>
+      <c r="B12" s="25" t="inlineStr">
+        <is>
+          <t>1m engineering sample (deductible)</t>
+        </is>
+      </c>
+      <c r="C12" s="24" t="n">
+        <v>1</v>
+      </c>
+      <c r="D12" s="24" t="inlineStr">
+        <is>
+          <t>pc</t>
+        </is>
+      </c>
+      <c r="E12" s="24" t="n">
+        <v>24</v>
+      </c>
+      <c r="F12" s="24" t="n">
+        <v>24</v>
+      </c>
+      <c r="G12" s="24" t="inlineStr">
+        <is>
+          <t>with neon</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="26" t="inlineStr">
+        <is>
+          <t>TOTAL USD (one 30m circuit illustration)</t>
+        </is>
+      </c>
+      <c r="B13" s="27" t="n"/>
+      <c r="C13" s="27" t="n"/>
+      <c r="D13" s="27" t="n"/>
+      <c r="E13" s="27" t="n"/>
+      <c r="F13" s="27" t="n">
+        <v>254.61</v>
+      </c>
+      <c r="G13" s="27" t="n"/>
+    </row>
+    <row r="15" ht="40" customHeight="1">
+      <c r="A15" s="31" t="inlineStr">
+        <is>
+          <t>Pricing note: Almaty retail mid silicone/architectural neon ≈ 2,500–3,500 KZT/m (≈USD 5.6–7.9 shelf). EXW 6.20 leaves partner room after freight/VAT to sell project package above local stock but far below typical Philips facade system cost. Drivers/DALI excluded.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="4">
+    <mergeCell ref="A13:D13"/>
+    <mergeCell ref="A2:G2"/>
+    <mergeCell ref="A1:G1"/>
+    <mergeCell ref="A15:G15"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:F50"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -1363,8 +2387,8 @@
   </sheetData>
   <mergeCells count="21">
     <mergeCell ref="A27:F27"/>
+    <mergeCell ref="A50:F50"/>
     <mergeCell ref="A18:F18"/>
-    <mergeCell ref="A50:F50"/>
     <mergeCell ref="A26:F26"/>
     <mergeCell ref="A21:F21"/>
     <mergeCell ref="A2:F2"/>
@@ -1388,7 +2412,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -1716,9 +2740,9 @@
           <t>TOTAL USD (illustration: one 30m circuit + clips + sample)</t>
         </is>
       </c>
-      <c r="B15" s="27" t="n"/>
-      <c r="C15" s="27" t="n"/>
-      <c r="D15" s="27" t="n"/>
+      <c r="B15" s="46" t="n"/>
+      <c r="C15" s="46" t="n"/>
+      <c r="D15" s="47" t="n"/>
       <c r="E15" s="27" t="n"/>
       <c r="F15" s="28" t="n">
         <v>296.03</v>
@@ -1769,7 +2793,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>

</xml_diff>